<commit_message>
Ap Voucher Advance and Document Payment along with ReferenceSitewiseFIFOsetoff for AP Voucher(Tested)
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/ApVoucher.xlsx
+++ b/src/test/resources/Finance/ApVoucher.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="2"/>
+    <workbookView windowWidth="20490" windowHeight="7620" firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="65">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -73,55 +73,73 @@
     <t>Ref1t54rf</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>LineNo</t>
+  </si>
+  <si>
+    <t>Sub Ledger</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>General Ledger</t>
+  </si>
+  <si>
+    <t>Reference Site</t>
+  </si>
+  <si>
+    <t>Ledger Narration</t>
+  </si>
+  <si>
+    <t>Is Reversal</t>
+  </si>
+  <si>
+    <t>Amount(Dr)</t>
+  </si>
+  <si>
+    <t>AdjustmentType</t>
+  </si>
+  <si>
+    <t>PaymentSelection</t>
+  </si>
+  <si>
+    <t>Deduct TDS</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>ABUL KASHEM MOLLHA</t>
+  </si>
+  <si>
+    <t>J061</t>
+  </si>
+  <si>
+    <t>Sundry Creditors for Expenses</t>
+  </si>
+  <si>
+    <t>Reference Site wise FIFO set-off</t>
+  </si>
+  <si>
+    <t>FIN-AP-ADV-TDS-EQ</t>
+  </si>
+  <si>
+    <t>AARUCHI FASHIONS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Sundry Creditors for Goods</t>
+  </si>
+  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>LineNo</t>
-  </si>
-  <si>
-    <t>Sub Ledger</t>
-  </si>
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>General Ledger</t>
-  </si>
-  <si>
-    <t>Reference Site</t>
-  </si>
-  <si>
-    <t>Ledger Narration</t>
-  </si>
-  <si>
-    <t>Is Reversal</t>
-  </si>
-  <si>
-    <t>Amount(Dr)</t>
-  </si>
-  <si>
-    <t>AdjustmentType</t>
-  </si>
-  <si>
-    <t>PaymentSelection</t>
-  </si>
-  <si>
-    <t>Deduct TDS</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>AARUCHI FASHIONS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>BT56</t>
-  </si>
-  <si>
-    <t>Sundry Creditors for Expenses</t>
-  </si>
-  <si>
-    <t>Cheque</t>
+    <t>FIN-AP-ADV-TDS-PE</t>
+  </si>
+  <si>
+    <t>FIN-AP-ADV-TDS-CEPT</t>
   </si>
   <si>
     <t>Payment Mode</t>
@@ -154,6 +172,9 @@
     <t>Adjustment Amount</t>
   </si>
   <si>
+    <t>TC102</t>
+  </si>
+  <si>
     <t>ECOM/00205/24-25</t>
   </si>
   <si>
@@ -178,6 +199,9 @@
     <t>Reference Site Name</t>
   </si>
   <si>
+    <t>Site Name</t>
+  </si>
+  <si>
     <t>TDS Name</t>
   </si>
   <si>
@@ -188,18 +212,34 @@
   </si>
   <si>
     <t>Populate TDS Exception Rate</t>
+  </si>
+  <si>
+    <t>TDS Applicable Amount Behaviour</t>
+  </si>
+  <si>
+    <t>TDS ON COMMISSION(678)</t>
+  </si>
+  <si>
+    <t>GROSS_EQUALS_TDS</t>
+  </si>
+  <si>
+    <t>PARTIAL_EDIT</t>
+  </si>
+  <si>
+    <t>CLEAR_ERROR_THEN_PARTIAL_EDIT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="181" formatCode="yyyy/mm/dd"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -222,15 +262,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF0A0A0A"/>
+      <sz val="9.8"/>
+      <color rgb="FF067D17"/>
       <name val="Courier New"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Courier New"/>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
@@ -680,178 +720,167 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -906,221 +935,7 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color theme="4"/>
-        </left>
-        <right style="thin">
-          <color theme="4"/>
-        </right>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-        <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-  </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
-    </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
-    </tableStyle>
-  </tableStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1390,6 +1205,7 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
+    <col min="1" max="1" width="22.7142857142857" customWidth="1"/>
     <col min="2" max="2" width="17.7142857142857" style="1" customWidth="1"/>
     <col min="3" max="3" width="15.7142857142857" style="1" customWidth="1"/>
     <col min="4" max="4" width="25.8571428571429" style="1" customWidth="1"/>
@@ -1408,7 +1224,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -1437,7 +1253,7 @@
       <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="9">
         <v>46165</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -1456,8 +1272,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1"/>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
     <col min="3" max="3" width="37.2857142857143" style="1" customWidth="1"/>
     <col min="4" max="4" width="29.7142857142857" style="1" customWidth="1"/>
@@ -1466,8 +1282,9 @@
     <col min="7" max="7" width="17.2857142857143" customWidth="1"/>
     <col min="8" max="8" width="12.2857142857143" style="1" customWidth="1"/>
     <col min="9" max="9" width="32.4285714285714" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.4285714285714" customWidth="1"/>
+    <col min="10" max="10" width="41.7142857142857" customWidth="1"/>
     <col min="11" max="11" width="18.7142857142857" customWidth="1"/>
+    <col min="12" max="12" width="11.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1515,24 +1332,101 @@
       <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>28</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
       </c>
       <c r="I2">
-        <v>2000</v>
-      </c>
-      <c r="J2" s="8"/>
-      <c r="K2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="1">
+        <v>217</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1940</v>
+      </c>
+      <c r="L3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="1">
+        <v>217</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1940</v>
+      </c>
+      <c r="L4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="1">
+        <v>217</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1940</v>
+      </c>
+      <c r="L5" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1544,8 +1438,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="6"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="11.4285714285714" style="1" customWidth="1"/>
     <col min="2" max="2" width="7.85714285714286" style="1" customWidth="1"/>
@@ -1564,36 +1458,19 @@
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2">
-        <v>455352</v>
-      </c>
-      <c r="E2" s="5">
-        <v>46165</v>
       </c>
     </row>
   </sheetData>
@@ -1624,42 +1501,42 @@
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H1" t="s">
         <v>18</v>
       </c>
       <c r="I1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="4">
         <v>45609</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>41</v>
+      <c r="E2" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="I2">
         <v>450</v>
@@ -1667,19 +1544,19 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="4">
         <v>45609</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>41</v>
+      <c r="E3" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="I3">
         <v>450</v>
@@ -1687,19 +1564,19 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="3">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4">
         <v>45609</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>41</v>
+      <c r="E4" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="I4">
         <v>900</v>
@@ -1707,19 +1584,19 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="3">
+      <c r="C5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="4">
         <v>46128</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>46</v>
+      <c r="E5" s="3" t="s">
+        <v>53</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -1734,22 +1611,45 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="2" width="21.5714285714286" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="4" width="21.5714285714286" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7142857142857" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
-        <v>39</v>
+      <c r="E1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1761,16 +1661,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="10.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="14.2857142857143" customWidth="1"/>
     <col min="3" max="3" width="23.8571428571429" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="5" max="5" width="23.8571428571429" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1778,16 +1680,99 @@
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
         <v>51</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2">
+        <v>2000</v>
+      </c>
+      <c r="E2">
+        <v>2000</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>1940</v>
+      </c>
+      <c r="E3">
+        <v>1940</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>1940</v>
+      </c>
+      <c r="E4">
+        <v>900</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5">
+        <v>1940</v>
+      </c>
+      <c r="E5">
+        <v>900</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>